<commit_message>
feat: sync local changes - medical insurance fix, payroll, attendance, leaves, salary config, employees, CMS, settings, developer module, dashboard widgets
</commit_message>
<xml_diff>
--- a/Templates/employee.xlsx
+++ b/Templates/employee.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HR_Erp_vscode\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDF2F985-3553-4EBC-8025-951B67B99EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0146D8F0-D2B9-43E6-9D28-D2E634D605E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="105">
   <si>
     <t>Employee Code</t>
   </si>
@@ -77,16 +77,280 @@
   </si>
   <si>
     <t>Code</t>
+  </si>
+  <si>
+    <t>Uncle Hefny</t>
+  </si>
+  <si>
+    <t>Ahmed Abdel Fattah</t>
+  </si>
+  <si>
+    <t>Ahmed Ehab kamal Abdallah</t>
+  </si>
+  <si>
+    <t>Ahmed Mohamed Badr Ahmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alaa  Ahmed abdelmoniam mohamed </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amal Mohamed ellithy </t>
+  </si>
+  <si>
+    <t>Arwa Osama Hassan Abdullah</t>
+  </si>
+  <si>
+    <t>Basma Seif El Dawla Hussien Hussien</t>
+  </si>
+  <si>
+    <t>Bothina khaled Mohamed abdelsattar</t>
+  </si>
+  <si>
+    <t>Dina Hossam Sayed Saleh Hassan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Eman Yousri </t>
+  </si>
+  <si>
+    <t>Eman Mohamed Ezat Shebl</t>
+  </si>
+  <si>
+    <t>Engy metwaly omar</t>
+  </si>
+  <si>
+    <t>Farah Abdelhakeem Sleem Wahby Mostafa</t>
+  </si>
+  <si>
+    <t>Flourance Atef Aziz</t>
+  </si>
+  <si>
+    <t>Royal</t>
+  </si>
+  <si>
+    <t>Rania El Laithy</t>
+  </si>
+  <si>
+    <t>Radwa Badr</t>
+  </si>
+  <si>
+    <t>Top Management</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Finance</t>
+  </si>
+  <si>
+    <t>Academic</t>
+  </si>
+  <si>
+    <t>Helpers</t>
+  </si>
+  <si>
+    <t>Medical</t>
+  </si>
+  <si>
+    <t>CEO</t>
+  </si>
+  <si>
+    <t>Executive Director</t>
+  </si>
+  <si>
+    <t>Financial Consultant</t>
+  </si>
+  <si>
+    <t>Photographer</t>
+  </si>
+  <si>
+    <t>Junior Accountant</t>
+  </si>
+  <si>
+    <t>Quran</t>
+  </si>
+  <si>
+    <t>Art teacher</t>
+  </si>
+  <si>
+    <t>Floor &amp; Helper Supervisor</t>
+  </si>
+  <si>
+    <t>Support Teacher</t>
+  </si>
+  <si>
+    <t>Arabic Teacher</t>
+  </si>
+  <si>
+    <t>Class Teacher</t>
+  </si>
+  <si>
+    <t>Part Time-Doctor</t>
+  </si>
+  <si>
+    <t>Music Teacher</t>
+  </si>
+  <si>
+    <t>Teacher</t>
+  </si>
+  <si>
+    <t>Marketing Representative</t>
+  </si>
+  <si>
+    <t>High Management</t>
+  </si>
+  <si>
+    <t>Part Time</t>
+  </si>
+  <si>
+    <t>Management</t>
+  </si>
+  <si>
+    <t>Part time</t>
+  </si>
+  <si>
+    <t>White Collar</t>
+  </si>
+  <si>
+    <t>Hager Tharwat Abdelghani Afifi</t>
+  </si>
+  <si>
+    <t>Heba Mohamed Medhat Mahmoud  Afifi</t>
+  </si>
+  <si>
+    <t>Jihan Mohamed Samir</t>
+  </si>
+  <si>
+    <t>Maha Safwat</t>
+  </si>
+  <si>
+    <t>Mayar Osama Hassan Abdallah</t>
+  </si>
+  <si>
+    <t>Mohamed Anwar (Captin)</t>
+  </si>
+  <si>
+    <t>Mohamed Mahmoud Sabry</t>
+  </si>
+  <si>
+    <t>Sherif</t>
+  </si>
+  <si>
+    <t>Nevine Mohamed Elsaid Ahmed Elbahiry</t>
+  </si>
+  <si>
+    <t>Nisreen Samir Mahrous Abdel Rehim</t>
+  </si>
+  <si>
+    <t>Nourhan Mahmoud Hussein Fouad</t>
+  </si>
+  <si>
+    <t>Osama Fathalla Mahmoud</t>
+  </si>
+  <si>
+    <t>Ramadan Shawky</t>
+  </si>
+  <si>
+    <t>Rana Ali Roushdy</t>
+  </si>
+  <si>
+    <t>Rania Salah Eldin Abdelaleam Elsayed</t>
+  </si>
+  <si>
+    <t>rasha moftah ahmed</t>
+  </si>
+  <si>
+    <t>Rawan Sherif</t>
+  </si>
+  <si>
+    <t>Sahar Ibrahim Elraie</t>
+  </si>
+  <si>
+    <t>Samar Elraei (Teacher)</t>
+  </si>
+  <si>
+    <t>Samar Ibrahim Mohamed Abdulaty Helal</t>
+  </si>
+  <si>
+    <t>Sarah Gad Abou Elmaaty</t>
+  </si>
+  <si>
+    <t>Yousra Emad Farouk</t>
+  </si>
+  <si>
+    <t>Ziad</t>
+  </si>
+  <si>
+    <t>Kattameya</t>
+  </si>
+  <si>
+    <t>Blue Collar</t>
+  </si>
+  <si>
+    <t>HR Manager</t>
+  </si>
+  <si>
+    <t>CO- Teacher</t>
+  </si>
+  <si>
+    <t>Stock Keeper</t>
+  </si>
+  <si>
+    <t>Part Time-Zumba Instructor</t>
+  </si>
+  <si>
+    <t>After School</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Security </t>
+  </si>
+  <si>
+    <t>Branch Manager</t>
+  </si>
+  <si>
+    <t>Academic Director</t>
+  </si>
+  <si>
+    <t>Financial Manager</t>
+  </si>
+  <si>
+    <t>Pe Head</t>
+  </si>
+  <si>
+    <t>Education Head</t>
+  </si>
+  <si>
+    <t>Events Manager</t>
+  </si>
+  <si>
+    <t>Purchases &amp; Maintenance</t>
+  </si>
+  <si>
+    <t>Purchasing</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Human Resources</t>
+  </si>
+  <si>
+    <t>Administration</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -457,15 +721,15 @@
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.875" customWidth="1"/>
-    <col min="4" max="4" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.25" customWidth="1"/>
+    <col min="4" max="4" width="26.375" customWidth="1"/>
     <col min="5" max="5" width="18.875" customWidth="1"/>
     <col min="6" max="6" width="11.25" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.375" customWidth="1"/>
-    <col min="11" max="11" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.75" customWidth="1"/>
+    <col min="10" max="10" width="32.375" customWidth="1"/>
+    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="5.875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.375" customWidth="1"/>
     <col min="14" max="14" width="8" bestFit="1" customWidth="1"/>
@@ -536,282 +800,1002 @@
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>10001</v>
+      </c>
       <c r="B2" t="str">
         <f>"EMP-"&amp;A2</f>
-        <v>EMP-</v>
+        <v>EMP-10001</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>10002</v>
+      </c>
       <c r="B3" t="str">
         <f t="shared" ref="B3:B66" si="0">"EMP-"&amp;A3</f>
-        <v>EMP-</v>
+        <v>EMP-10002</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>10005</v>
+      </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10005</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K4" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>10491</v>
+      </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10491</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" t="s">
+        <v>46</v>
+      </c>
+      <c r="K5" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>10473</v>
+      </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10473</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" t="s">
+        <v>47</v>
+      </c>
+      <c r="K6" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>10477</v>
+      </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10477</v>
+      </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+      <c r="I7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J7" t="s">
+        <v>48</v>
+      </c>
+      <c r="K7" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>10169</v>
+      </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10169</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J8" t="s">
+        <v>49</v>
+      </c>
+      <c r="K8" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>10334</v>
+      </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10334</v>
+      </c>
+      <c r="C9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" t="s">
+        <v>34</v>
+      </c>
+      <c r="I9" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9" t="s">
+        <v>50</v>
+      </c>
+      <c r="K9" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>10484</v>
+      </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10484</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10" t="s">
+        <v>40</v>
+      </c>
+      <c r="J10" t="s">
+        <v>51</v>
+      </c>
+      <c r="K10" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10482</v>
+      </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10482</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J11" t="s">
+        <v>52</v>
+      </c>
+      <c r="K11" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>10428</v>
+      </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10428</v>
+      </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+      <c r="H12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" t="s">
+        <v>40</v>
+      </c>
+      <c r="J12" t="s">
+        <v>53</v>
+      </c>
+      <c r="K12" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>10012</v>
+      </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10012</v>
+      </c>
+      <c r="C13" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I13" t="s">
+        <v>40</v>
+      </c>
+      <c r="J13" t="s">
+        <v>52</v>
+      </c>
+      <c r="K13" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>10014</v>
+      </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10014</v>
+      </c>
+      <c r="C14" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" t="s">
+        <v>34</v>
+      </c>
+      <c r="I14" t="s">
+        <v>42</v>
+      </c>
+      <c r="J14" t="s">
+        <v>54</v>
+      </c>
+      <c r="K14" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>10187</v>
+      </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
+        <v>EMP-10187</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+      <c r="H15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" t="s">
+        <v>40</v>
+      </c>
+      <c r="J15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K15" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>10429</v>
+      </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10429</v>
+      </c>
+      <c r="C16" t="s">
+        <v>31</v>
+      </c>
+      <c r="H16" t="s">
+        <v>34</v>
+      </c>
+      <c r="I16" t="s">
+        <v>40</v>
+      </c>
+      <c r="J16" t="s">
+        <v>53</v>
+      </c>
+      <c r="K16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>10483</v>
+      </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10483</v>
+      </c>
+      <c r="C17" t="s">
+        <v>32</v>
+      </c>
+      <c r="H17" t="s">
+        <v>34</v>
+      </c>
+      <c r="I17" t="s">
+        <v>40</v>
+      </c>
+      <c r="J17" t="s">
+        <v>56</v>
+      </c>
+      <c r="K17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>10145</v>
+      </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10145</v>
+      </c>
+      <c r="C18" t="s">
+        <v>33</v>
+      </c>
+      <c r="H18" t="s">
+        <v>34</v>
+      </c>
+      <c r="I18" t="s">
+        <v>38</v>
+      </c>
+      <c r="J18" t="s">
+        <v>57</v>
+      </c>
+      <c r="K18" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>10479</v>
+      </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10479</v>
+      </c>
+      <c r="C19" t="s">
+        <v>63</v>
+      </c>
+      <c r="H19" t="s">
+        <v>34</v>
+      </c>
+      <c r="I19" t="s">
+        <v>40</v>
+      </c>
+      <c r="J19" t="s">
+        <v>89</v>
+      </c>
+      <c r="K19" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>10017</v>
+      </c>
       <c r="B20" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10017</v>
+      </c>
+      <c r="C20" t="s">
+        <v>64</v>
+      </c>
+      <c r="H20" t="s">
+        <v>34</v>
+      </c>
+      <c r="I20" t="s">
+        <v>40</v>
+      </c>
+      <c r="J20" t="s">
+        <v>95</v>
+      </c>
+      <c r="K20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>10402</v>
+      </c>
       <c r="B21" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10402</v>
+      </c>
+      <c r="C21" t="s">
+        <v>65</v>
+      </c>
+      <c r="H21" t="s">
+        <v>34</v>
+      </c>
+      <c r="I21" t="s">
+        <v>101</v>
+      </c>
+      <c r="J21" t="s">
+        <v>90</v>
+      </c>
+      <c r="K21" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>10315</v>
+      </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10315</v>
+      </c>
+      <c r="C22" t="s">
+        <v>66</v>
+      </c>
+      <c r="H22" t="s">
+        <v>34</v>
+      </c>
+      <c r="I22" t="s">
+        <v>38</v>
+      </c>
+      <c r="J22" t="s">
+        <v>57</v>
+      </c>
+      <c r="K22" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22101</v>
+      </c>
       <c r="B23" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-22101</v>
+      </c>
+      <c r="C23" t="s">
+        <v>67</v>
+      </c>
+      <c r="H23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I23" t="s">
+        <v>40</v>
+      </c>
+      <c r="J23" t="s">
+        <v>53</v>
+      </c>
+      <c r="K23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>10011</v>
+      </c>
       <c r="B24" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10011</v>
+      </c>
+      <c r="C24" t="s">
+        <v>68</v>
+      </c>
+      <c r="H24" t="s">
+        <v>34</v>
+      </c>
+      <c r="I24" t="s">
+        <v>40</v>
+      </c>
+      <c r="J24" t="s">
+        <v>91</v>
+      </c>
+      <c r="K24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>10497</v>
+      </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10497</v>
+      </c>
+      <c r="C25" t="s">
+        <v>69</v>
+      </c>
+      <c r="H25" t="s">
+        <v>34</v>
+      </c>
+      <c r="I25" t="s">
+        <v>103</v>
+      </c>
+      <c r="J25" t="s">
+        <v>88</v>
+      </c>
+      <c r="K25" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>10006</v>
+      </c>
       <c r="B26" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10006</v>
+      </c>
+      <c r="C26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H26" t="s">
+        <v>34</v>
+      </c>
+      <c r="I26" t="s">
+        <v>39</v>
+      </c>
+      <c r="J26" t="s">
+        <v>96</v>
+      </c>
+      <c r="K26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>10452</v>
+      </c>
       <c r="B27" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10452</v>
+      </c>
+      <c r="C27" t="s">
+        <v>71</v>
+      </c>
+      <c r="H27" t="s">
+        <v>34</v>
+      </c>
+      <c r="I27" t="s">
+        <v>40</v>
+      </c>
+      <c r="J27" t="s">
+        <v>53</v>
+      </c>
+      <c r="K27" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>10463</v>
+      </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10463</v>
+      </c>
+      <c r="C28" t="s">
+        <v>72</v>
+      </c>
+      <c r="H28" t="s">
+        <v>34</v>
+      </c>
+      <c r="I28" t="s">
+        <v>40</v>
+      </c>
+      <c r="J28" t="s">
+        <v>53</v>
+      </c>
+      <c r="K28" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>10439</v>
+      </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10439</v>
+      </c>
+      <c r="C29" t="s">
+        <v>73</v>
+      </c>
+      <c r="H29" t="s">
+        <v>34</v>
+      </c>
+      <c r="I29" t="s">
+        <v>104</v>
+      </c>
+      <c r="J29" t="s">
+        <v>92</v>
+      </c>
+      <c r="K29" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>10248</v>
+      </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10248</v>
+      </c>
+      <c r="C30" t="s">
+        <v>74</v>
+      </c>
+      <c r="H30" t="s">
+        <v>34</v>
+      </c>
+      <c r="I30" t="s">
+        <v>40</v>
+      </c>
+      <c r="J30" t="s">
+        <v>97</v>
+      </c>
+      <c r="K30" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>10488</v>
+      </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10488</v>
+      </c>
+      <c r="C31" t="s">
+        <v>75</v>
+      </c>
+      <c r="H31" t="s">
+        <v>34</v>
+      </c>
+      <c r="I31" t="s">
+        <v>102</v>
+      </c>
+      <c r="J31" t="s">
+        <v>93</v>
+      </c>
+      <c r="K31" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>10019</v>
+      </c>
       <c r="B32" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10019</v>
+      </c>
+      <c r="C32" t="s">
+        <v>76</v>
+      </c>
+      <c r="H32" t="s">
+        <v>34</v>
+      </c>
+      <c r="I32" t="s">
+        <v>40</v>
+      </c>
+      <c r="J32" t="s">
+        <v>53</v>
+      </c>
+      <c r="K32" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>10449</v>
+      </c>
       <c r="B33" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10449</v>
+      </c>
+      <c r="C33" t="s">
+        <v>77</v>
+      </c>
+      <c r="H33" t="s">
+        <v>34</v>
+      </c>
+      <c r="I33" t="s">
+        <v>40</v>
+      </c>
+      <c r="J33" t="s">
+        <v>89</v>
+      </c>
+      <c r="K33" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>10043</v>
+      </c>
       <c r="B34" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10043</v>
+      </c>
+      <c r="C34" t="s">
+        <v>78</v>
+      </c>
+      <c r="H34" t="s">
+        <v>34</v>
+      </c>
+      <c r="I34" t="s">
+        <v>40</v>
+      </c>
+      <c r="J34" t="s">
+        <v>89</v>
+      </c>
+      <c r="K34" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>10472</v>
+      </c>
       <c r="B35" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10472</v>
+      </c>
+      <c r="C35" t="s">
+        <v>79</v>
+      </c>
+      <c r="H35" t="s">
+        <v>34</v>
+      </c>
+      <c r="I35" t="s">
+        <v>40</v>
+      </c>
+      <c r="J35" t="s">
+        <v>98</v>
+      </c>
+      <c r="K35" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>10101</v>
+      </c>
       <c r="B36" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10101</v>
+      </c>
+      <c r="C36" t="s">
+        <v>80</v>
+      </c>
+      <c r="H36" t="s">
+        <v>34</v>
+      </c>
+      <c r="I36" t="s">
+        <v>60</v>
+      </c>
+      <c r="J36" t="s">
+        <v>99</v>
+      </c>
+      <c r="K36" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>10018</v>
+      </c>
       <c r="B37" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10018</v>
+      </c>
+      <c r="C37" t="s">
+        <v>81</v>
+      </c>
+      <c r="H37" t="s">
+        <v>34</v>
+      </c>
+      <c r="I37" t="s">
+        <v>40</v>
+      </c>
+      <c r="J37" t="s">
+        <v>53</v>
+      </c>
+      <c r="K37" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>10475</v>
+      </c>
       <c r="B38" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10475</v>
+      </c>
+      <c r="C38" t="s">
+        <v>82</v>
+      </c>
+      <c r="H38" t="s">
+        <v>34</v>
+      </c>
+      <c r="I38" t="s">
+        <v>40</v>
+      </c>
+      <c r="J38" t="s">
+        <v>53</v>
+      </c>
+      <c r="K38" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>10121</v>
+      </c>
       <c r="B39" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10121</v>
+      </c>
+      <c r="C39" t="s">
+        <v>83</v>
+      </c>
+      <c r="H39" t="s">
+        <v>34</v>
+      </c>
+      <c r="I39" t="s">
+        <v>104</v>
+      </c>
+      <c r="J39" t="s">
+        <v>94</v>
+      </c>
+      <c r="K39" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>10217</v>
+      </c>
       <c r="B40" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10217</v>
+      </c>
+      <c r="C40" t="s">
+        <v>84</v>
+      </c>
+      <c r="H40" t="s">
+        <v>34</v>
+      </c>
+      <c r="I40" t="s">
+        <v>40</v>
+      </c>
+      <c r="J40" t="s">
+        <v>53</v>
+      </c>
+      <c r="K40" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>10008</v>
+      </c>
       <c r="B41" t="str">
         <f t="shared" si="0"/>
-        <v>EMP-</v>
-      </c>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+        <v>EMP-10008</v>
+      </c>
+      <c r="C41" t="s">
+        <v>85</v>
+      </c>
+      <c r="H41" t="s">
+        <v>34</v>
+      </c>
+      <c r="I41" t="s">
+        <v>104</v>
+      </c>
+      <c r="J41" t="s">
+        <v>100</v>
+      </c>
+      <c r="K41" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B42" t="str">
         <f t="shared" si="0"/>
         <v>EMP-</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B43" t="str">
         <f t="shared" si="0"/>
         <v>EMP-</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B44" t="str">
         <f t="shared" si="0"/>
         <v>EMP-</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B45" t="str">
         <f t="shared" si="0"/>
         <v>EMP-</v>
       </c>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B46" t="str">
         <f t="shared" si="0"/>
         <v>EMP-</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B47" t="str">
         <f t="shared" si="0"/>
         <v>EMP-</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B48" t="str">
         <f t="shared" si="0"/>
         <v>EMP-</v>
@@ -1730,6 +2714,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError sqref="B1:S1" numberStoredAsText="1"/>

</xml_diff>